<commit_message>
more playing around with examples
</commit_message>
<xml_diff>
--- a/wombat_Y2SiO5_example/reciprocal_space_conversion_Y2SiO5.xlsx
+++ b/wombat_Y2SiO5_example/reciprocal_space_conversion_Y2SiO5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\wombat_instrument_work\eulerian_cradle\Wombat_DMCpy\wombat_Y2SiO5_example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0DB067-2416-4887-B273-FF2928637730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D506A0-2853-4D44-B1C8-0290344DB2CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26760" yWindow="2160" windowWidth="21600" windowHeight="12510" activeTab="1" xr2:uid="{1785FB5C-C68B-4CD0-A3EB-01061EC28F90}"/>
+    <workbookView xWindow="-25650" yWindow="4545" windowWidth="21600" windowHeight="12510" activeTab="1" xr2:uid="{1785FB5C-C68B-4CD0-A3EB-01061EC28F90}"/>
   </bookViews>
   <sheets>
     <sheet name="2theta_to_Q" sheetId="2" r:id="rId1"/>
@@ -118,12 +118,18 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -138,8 +144,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,13 +595,13 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="1">
         <v>-6.4000000000000001E-2</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="1">
         <v>2.145</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="1">
         <v>-5.0000000000000001E-3</v>
       </c>
       <c r="D5">
@@ -609,24 +616,24 @@
         <f>DEGREES(2*ASIN($F$2/(2*E5)))</f>
         <v>48.605228839417563</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="1">
         <v>2</v>
       </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="1">
         <v>-3.972</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="1">
         <v>-1.7649999999999999</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="1">
         <v>-0.15490000000000001</v>
       </c>
       <c r="D6">
@@ -641,13 +648,13 @@
         <f>DEGREES(2*ASIN($F$2/(2*E6)))</f>
         <v>113.0459740830986</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="1">
         <v>4</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
         <v>-4</v>
       </c>
     </row>
@@ -716,17 +723,35 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>-4.47</v>
+      </c>
+      <c r="B9">
+        <v>-0.27189999999999998</v>
+      </c>
+      <c r="C9">
+        <v>0.317</v>
+      </c>
       <c r="D9">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="E9" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F9" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>4.4894675196508551</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>1.399539094486695</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="2"/>
+        <v>118.85758906897046</v>
+      </c>
+      <c r="H9">
+        <v>10</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>-4</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>